<commit_message>
#4 #3 ZX-SH1.0-4PWT Updated in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/LED Board - v1.0/BOM/Client-BOM-LED Board-v1.0.xlsx
+++ b/Design Files/LED Board - v1.0/BOM/Client-BOM-LED Board-v1.0.xlsx
@@ -66,9 +66,6 @@
     <t>CAP CER 0.1UF 25V X5R 0402</t>
   </si>
   <si>
-    <t>CONN HEADER SMD R/A 4POS 1MM</t>
-  </si>
-  <si>
     <t>SMD5050 Light Emitting Diodes (LED) ROHS</t>
   </si>
   <si>
@@ -84,9 +81,6 @@
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>SM04B-SRSS-TB(LF)(SN)</t>
-  </si>
-  <si>
     <t>WS2812B-XF02/W</t>
   </si>
   <si>
@@ -139,6 +133,12 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>ZX-SH1.0-4PWT</t>
+  </si>
+  <si>
+    <t>1x4P 4P 1 SH 1mm Tin 4 -25℃~+85℃ Brass 1A Horizontal attachment SMD,P=1mm,Surface Mount，Right Angle Wire To Board Connector ROHS</t>
   </si>
 </sst>
 </file>
@@ -674,22 +674,22 @@
         <v>13</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -708,23 +708,23 @@
         <v>14</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J3" s="7">
         <v>3</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B6" si="0">ROW(B4) - ROW($B$2)</f>
@@ -737,19 +737,19 @@
         <v>9</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>21</v>
-      </c>
       <c r="H4" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -769,19 +769,19 @@
         <v>10</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
@@ -801,19 +801,19 @@
         <v>11</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -833,19 +833,19 @@
         <v>12</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>

</xml_diff>